<commit_message>
Rewrite README around four KPIs; import human review of shipped run
- README: human, story-first voice; four KPIs with thresholds and the
  reasoning behind each; three-system trade-off; lessons learned.
- Case study: KPI section with targets, updated shipped-run figures.
- Human review of 35fe63c2 overturns 4 judge scores (2 correctness,
  2 groundedness): correctness 0.878 -> 0.927, groundedness 0.927 -> 0.976.
  Lessons recorded in evals/human_labels.json.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/eval-sheets/eval_all_eu-ai-act-agentic-reflect-35fe63c2.xlsx
+++ b/results/eval-sheets/eval_all_eu-ai-act-agentic-reflect-35fe63c2.xlsx
@@ -30,12 +30,18 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+        <bgColor rgb="00BDD7EE"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -56,13 +62,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -941,13 +950,13 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>1</v>
@@ -1137,12 +1146,12 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="2" t="n">
@@ -1580,10 +1589,10 @@
       <c r="H12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="3" t="n">
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K12" s="2" t="n">
@@ -1685,7 +1694,7 @@
       <c r="H13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="I13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="2" t="n">
@@ -2136,7 +2145,7 @@
       <c r="I18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="3" t="n">
+      <c r="J18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K18" s="2" t="n">
@@ -2205,16 +2214,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F19" s="3" t="n">
+      <c r="F19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="3" t="n">
+      <c r="H19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="2" t="n">
@@ -2676,7 +2685,7 @@
       <c r="H24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I24" s="3" t="n">
+      <c r="I24" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="2" t="n">
@@ -3427,7 +3436,7 @@
         <v>1</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" s="2" t="n">
         <v>1</v>
@@ -4000,7 +4009,7 @@
       <c r="G39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H39" s="3" t="n">
+      <c r="H39" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="2" t="n">
@@ -4321,7 +4330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4351,7 +4360,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.927</v>
+        <v>0.976</v>
       </c>
       <c r="C2" t="n">
         <v>41</v>
@@ -4377,7 +4386,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.878</v>
+        <v>0.927</v>
       </c>
       <c r="C4" t="n">
         <v>41</v>
@@ -4386,76 +4395,76 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>retrieval (strict)</t>
+          <t>groundedness (judge only, before human review)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.895</v>
+        <v>0.927</v>
       </c>
       <c r="C5" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>top-3 citation hit</t>
+          <t>answer_relevance (judge only, before human review)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.944</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>recall@1</t>
+          <t>answer_correctness (judge only, before human review)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.394</v>
+        <v>0.878</v>
       </c>
       <c r="C7" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>recall@3</t>
+          <t>judge-human agreement</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.833</v>
+        <v>0.967</v>
       </c>
       <c r="C8" t="n">
-        <v>36</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>recall@5</t>
+          <t>retrieval (strict)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.898</v>
+        <v>0.895</v>
       </c>
       <c r="C9" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>recall@8</t>
+          <t>top-3 citation hit</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.944</v>
       </c>
       <c r="C10" t="n">
         <v>36</v>
@@ -4464,11 +4473,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>precision@1 (lower bound)</t>
+          <t>recall@1</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.5</v>
+        <v>0.394</v>
       </c>
       <c r="C11" t="n">
         <v>36</v>
@@ -4477,11 +4486,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>precision@3 (lower bound)</t>
+          <t>recall@3</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.472</v>
+        <v>0.833</v>
       </c>
       <c r="C12" t="n">
         <v>36</v>
@@ -4490,11 +4499,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>precision@5 (lower bound)</t>
+          <t>recall@5</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.361</v>
+        <v>0.898</v>
       </c>
       <c r="C13" t="n">
         <v>36</v>
@@ -4503,11 +4512,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>precision@8 (lower bound)</t>
+          <t>recall@8</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.288</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="C14" t="n">
         <v>36</v>
@@ -4516,47 +4525,99 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>latency s (mean)</t>
+          <t>precision@1 (lower bound)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.581</v>
+        <v>0.5</v>
       </c>
       <c r="C15" t="n">
-        <v>41</v>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>precision@3 (lower bound)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.472</v>
+      </c>
+      <c r="C16" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>experiment</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>eu-ai-act-agentic-reflect-35fe63c2</t>
-        </is>
+          <t>precision@5 (lower bound)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="C17" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LEGEND</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>blue judge cell = human override (evals/human_labels.json); pink = score 0</t>
-        </is>
+          <t>precision@8 (lower bound)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="C18" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>latency s (mean)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>15.581</v>
+      </c>
+      <c r="C19" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>experiment</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>eu-ai-act-agentic-reflect-35fe63c2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>LEGEND</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>blue judge cell = human override (evals/human_labels.json); pink = score 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Precision is a lower bound: the golden expected_source lists only primary sources. All averages are per-question (macro).</t>
         </is>

</xml_diff>